<commit_message>
결과 파일 업데이트 2026-08-25 08:35
</commit_message>
<xml_diff>
--- a/results/andar_할인율모니터링_20260825.xlsx
+++ b/results/andar_할인율모니터링_20260825.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H163"/>
+  <dimension ref="A1:H166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,7 +491,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3,456</t>
+          <t>3,459</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3,456</t>
+          <t>3,459</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>1,915</t>
+          <t>1,916</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1,915</t>
+          <t>1,916</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>1,915</t>
+          <t>1,916</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>66</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>9,994</t>
+          <t>9,996</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>96</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>5,063</t>
+          <t>5,064</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>699</t>
+          <t>700</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2,254</t>
+          <t>2,255</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1667,7 +1667,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>26,974</t>
+          <t>26,977</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>26,974</t>
+          <t>26,977</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>26,974</t>
+          <t>26,977</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>10,332</t>
+          <t>10,333</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>677</t>
+          <t>678</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>1,557</t>
+          <t>1,558</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>1,557</t>
+          <t>1,558</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>1,557</t>
+          <t>1,558</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>221</t>
+          <t>222</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>3,161</t>
+          <t>3,165</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>3,161</t>
+          <t>3,165</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>676</t>
+          <t>677</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>349</t>
+          <t>351</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>137</t>
+          <t>138</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4103,7 +4103,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>495</t>
+          <t>496</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -4145,7 +4145,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>495</t>
+          <t>496</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -4439,7 +4439,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>677</t>
+          <t>678</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -4481,7 +4481,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>555</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -7223,42 +7223,168 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17407&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16632&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>EPTBG-04</t>
+          <t>EPTSV-02</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>드라이 페더 버킷백</t>
+          <t>[1&amp;1] 하이 서포트 발목 보호대</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>55,000</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>104</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>https://andar.co.kr/product/detail.html?product_no=15151&amp;cate_no=2100&amp;display_group=1</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>EOTBG-22</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>투포켓 로고 캔버스백</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>49,000</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>49,000</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>https://andar.co.kr/product/detail.html?product_no=14561&amp;cate_no=2100&amp;display_group=1</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>EOTBG-05</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>메쉬 포켓 비치백</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>49,000</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>19,000</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>61%</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>https://andar.co.kr/product/detail.html?product_no=11110&amp;cate_no=2100&amp;display_group=1</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>ENTCP-01</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>와이드 셰이드 버킷햇</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>59,000</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>29,000</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>51%</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>681</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>4.7</t>
         </is>
       </c>
     </row>

</xml_diff>